<commit_message>
Added to Technical Assessment Questions
</commit_message>
<xml_diff>
--- a/technical_assessment_by_job/questions/docker_questions.xlsx
+++ b/technical_assessment_by_job/questions/docker_questions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_openai\codex_projects\technical_assessment_by_job\questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F617528-093A-40CD-A23C-1718F4A23735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6FCE41F-CA1C-423C-B453-0E5733CA2DB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="198">
   <si>
     <t>Question</t>
   </si>
@@ -554,13 +554,176 @@
   </si>
   <si>
     <t>By default, containers run as the 'root' user unless specified otherwise using the 'USER' instruction in the Dockerfile.</t>
+  </si>
+  <si>
+    <t>How do you choose a base image for a production-ready AWS CLI Docker image?</t>
+  </si>
+  <si>
+    <t>Use a minimal, stable base like debian:bookworm-slim or python:3.11-slim to reduce the attack surface and image size.</t>
+  </si>
+  <si>
+    <t>Why should you avoid running Docker containers as root?</t>
+  </si>
+  <si>
+    <t>If a container is compromised, root access inside the container can lead to host-level exploitation; always create a dedicated user.</t>
+  </si>
+  <si>
+    <t>It allows you to use a "build" stage to install dependencies and a "production" stage to copy only the final binary, keeping the final image lean.</t>
+  </si>
+  <si>
+    <t>What is a multi-stage build and why use it for the AWS CLI?</t>
+  </si>
+  <si>
+    <t>How do you handle secrets (like AWS keys) in a Dockerfile?</t>
+  </si>
+  <si>
+    <t>Never hardcode them; use environment variables at runtime or AWS IAM Roles/Task Roles instead of static keys.</t>
+  </si>
+  <si>
+    <t>How do you keep Docker image sizes small?</t>
+  </si>
+  <si>
+    <t>Chain commands with &amp;&amp;, delete package manager caches in the same layer, and use .dockerignore.</t>
+  </si>
+  <si>
+    <t>What is the difference between an entrypoint and a command (CMD)?</t>
+  </si>
+  <si>
+    <t>Entrypoint sets the executable; CMD provides default arguments that can be easily overridden.</t>
+  </si>
+  <si>
+    <t>How do you verify the integrity of the AWS CLI bundle you download in a Dockerfile?</t>
+  </si>
+  <si>
+    <t>By checking the GPG signature or checksum provided by Amazon against the downloaded file.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">What happens if you don't use </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>.dockerignore</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Large local files (like </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>.git</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or node_modules) are sent to the Docker daemon, slowing down builds and bloating the image.</t>
+    </r>
+  </si>
+  <si>
+    <t>How do you update the AWS CLI version in your image safely?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pin specific versions in the Dockerfile rather than using </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>latest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to ensure build reproducibility.</t>
+    </r>
+  </si>
+  <si>
+    <t>How do you troubleshoot a container that crashes immediately upon startup?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Check </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>docker logs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, use </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>docker inspect</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to verify the entrypoint, and try running the container with an interactive shell.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -575,6 +738,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -924,10 +1093,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="62.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="69" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="223.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1954,6 +2123,116 @@
         <v>101</v>
       </c>
     </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A94" s="2">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>178</v>
+      </c>
+      <c r="C94" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A95" s="2">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>180</v>
+      </c>
+      <c r="C95" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A96" s="2">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
+        <v>183</v>
+      </c>
+      <c r="C96" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A97" s="2">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>184</v>
+      </c>
+      <c r="C97" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A98" s="2">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>186</v>
+      </c>
+      <c r="C98" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A99" s="2">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
+        <v>188</v>
+      </c>
+      <c r="C99" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A100" s="2">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>190</v>
+      </c>
+      <c r="C100" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A101" s="2">
+        <v>100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>192</v>
+      </c>
+      <c r="C101" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A102" s="2">
+        <v>101</v>
+      </c>
+      <c r="B102" t="s">
+        <v>194</v>
+      </c>
+      <c r="C102" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A103" s="2">
+        <v>102</v>
+      </c>
+      <c r="B103" t="s">
+        <v>196</v>
+      </c>
+      <c r="C103" t="s">
+        <v>197</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>